<commit_message>
test: verifica las 12 hipotesis de defecto contra la instancia real
Ejecucion de comprobaciones dirigidas contra la demo publica para
confirmar cada sospecha antes de reportarla. Resultado: 6 confirmadas,
4 descartadas por comportamiento correcto y 2 no verificables por falta
de volumen de datos en el entorno.

Estados actualizados en la matriz: 29 Pasa, 6 Falla, 3 Bloqueado.
</commit_message>
<xml_diff>
--- a/02-casos-de-prueba.xlsx
+++ b/02-casos-de-prueba.xlsx
@@ -1305,14 +1305,14 @@
           <t>Tabla de decisión (R5)</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>Falla</t>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>BUG-002</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1563,14 +1563,14 @@
           <t>Conjetura de errores</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>Falla</t>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>BUG-003</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1822,14 +1822,14 @@
           <t>Valores límite</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>Falla</t>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>BUG-004</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1887,14 +1887,14 @@
           <t>Transición de estados</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>Falla</t>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>Bloqueado</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>BUG-005</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2340,14 +2340,14 @@
           <t>Particiones de equivalencia</t>
         </is>
       </c>
-      <c r="K28" s="7" t="inlineStr">
-        <is>
-          <t>Falla</t>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>BUG-007</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -2792,14 +2792,14 @@
           <t>Valores límite</t>
         </is>
       </c>
-      <c r="K35" s="7" t="inlineStr">
-        <is>
-          <t>Falla</t>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L35" s="6" t="inlineStr">
         <is>
-          <t>BUG-010</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3108,7 +3108,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
@@ -3118,7 +3118,7 @@
         </is>
       </c>
       <c r="B5" s="11" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -3128,7 +3128,7 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
docs: adjunta las evidencias reales y cierra la ultima hipotesis pendiente
Se capturan y embeben 13 capturas contra la instancia real. Cada
reporte confirmado pasa de una tabla de capturas pendientes a las
imagenes con su pie explicando que hay que mirar en cada una.

Al volver sobre el entorno, la instancia se habia repoblado de 4 a 188
empleados, lo que permitio ejecutar CP-020: la ordenacion SI se propaga
al paginar (sortField y sortOrder viajan en la peticion de la pagina
2). La hipotesis pasa de no verificable a descartada, con su evidencia.

CP-019 sigue bloqueado, ahora por un motivo mejor documentado: exige
que la ultima pagina tenga exactamente un registro, y forzarlo obligaria
a borrar 37 empleados de una demo compartida.

Totales del ciclo: 30 Pasa, 6 Falla, 2 Bloqueado. Cobertura de
ejecucion 94,7%. Veredicto APTO CON RESERVAS sin cambios.
</commit_message>
<xml_diff>
--- a/02-casos-de-prueba.xlsx
+++ b/02-casos-de-prueba.xlsx
@@ -1887,9 +1887,9 @@
           <t>Transición de estados</t>
         </is>
       </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>Bloqueado</t>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>Pasa</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -3108,7 +3108,7 @@
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -3128,7 +3128,7 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">

</xml_diff>